<commit_message>
Improve visual; fix several cluster names and groups
</commit_message>
<xml_diff>
--- a/interim/cluster_review.xlsx
+++ b/interim/cluster_review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ilya/spatial-queries/interim/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0EA87CF-2D7D-6744-8FA1-7520FC3CF05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28A8CFD-DAF4-DB49-ABE9-DC0F43293457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16760" yWindow="1700" windowWidth="32300" windowHeight="26900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="15120" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="457">
   <si>
     <t>label</t>
   </si>
@@ -1198,9 +1198,6 @@
     <t>Languages spoken</t>
   </si>
   <si>
-    <t>Continents &amp; world regions</t>
-  </si>
-  <si>
     <t>Plate tectonics</t>
   </si>
   <si>
@@ -1355,6 +1352,45 @@
   </si>
   <si>
     <t>Other</t>
+  </si>
+  <si>
+    <t>name_raw</t>
+  </si>
+  <si>
+    <t>group_raw</t>
+  </si>
+  <si>
+    <t>Administrative</t>
+  </si>
+  <si>
+    <t>Cultural</t>
+  </si>
+  <si>
+    <t>Physical</t>
+  </si>
+  <si>
+    <t>Historical</t>
+  </si>
+  <si>
+    <t>Statistical</t>
+  </si>
+  <si>
+    <t>Regions and countries</t>
+  </si>
+  <si>
+    <t>POIs &amp; Commercial</t>
+  </si>
+  <si>
+    <t>Temporal-spatial &amp; Events</t>
+  </si>
+  <si>
+    <t>Birthplaces &amp; residences</t>
+  </si>
+  <si>
+    <t>Schools attended</t>
+  </si>
+  <si>
+    <t>University admissions / tests</t>
   </si>
 </sst>
 </file>
@@ -1376,15 +1412,27 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1411,25 +1459,50 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
+      <right/>
+      <top style="thin">
         <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
       </right>
-      <top/>
-      <bottom/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1732,17 +1805,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="8.33203125" customWidth="1"/>
     <col min="4" max="4" width="26.5" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="29.6640625" customWidth="1"/>
-    <col min="7" max="7" width="22.1640625" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="22.1640625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="36.1640625" style="6" customWidth="1"/>
+    <col min="9" max="9" width="30.83203125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1755,17 +1830,23 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F1" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>-1</v>
       </c>
@@ -1781,11 +1862,14 @@
       <c r="E2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F2" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>0</v>
       </c>
@@ -1801,14 +1885,20 @@
       <c r="E3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="5" t="s">
         <v>323</v>
       </c>
-      <c r="G3" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G3" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1824,14 +1914,20 @@
       <c r="E4" t="s">
         <v>13</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="5" t="s">
         <v>324</v>
       </c>
-      <c r="G4" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G4" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2</v>
       </c>
@@ -1847,14 +1943,20 @@
       <c r="E5" t="s">
         <v>16</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="G5" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G5" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>3</v>
       </c>
@@ -1870,14 +1972,20 @@
       <c r="E6" t="s">
         <v>19</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="5" t="s">
         <v>326</v>
       </c>
-      <c r="G6" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G6" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>4</v>
       </c>
@@ -1893,14 +2001,20 @@
       <c r="E7" t="s">
         <v>22</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="G7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G7" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>5</v>
       </c>
@@ -1916,14 +2030,20 @@
       <c r="E8" t="s">
         <v>25</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>438</v>
       </c>
-      <c r="G8" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H8" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>6</v>
       </c>
@@ -1939,14 +2059,20 @@
       <c r="E9" t="s">
         <v>28</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="G9" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G9" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>7</v>
       </c>
@@ -1962,14 +2088,20 @@
       <c r="E10" t="s">
         <v>31</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="G10" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G10" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>8</v>
       </c>
@@ -1985,14 +2117,20 @@
       <c r="E11" t="s">
         <v>34</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="5" t="s">
         <v>330</v>
       </c>
-      <c r="G11" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G11" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>9</v>
       </c>
@@ -2008,14 +2146,20 @@
       <c r="E12" t="s">
         <v>37</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="G12" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G12" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>455</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>10</v>
       </c>
@@ -2031,14 +2175,20 @@
       <c r="E13" t="s">
         <v>40</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="G13" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G13" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>11</v>
       </c>
@@ -2054,14 +2204,20 @@
       <c r="E14" t="s">
         <v>43</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="G14" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G14" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>12</v>
       </c>
@@ -2077,14 +2233,20 @@
       <c r="E15" t="s">
         <v>46</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="G15" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G15" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>13</v>
       </c>
@@ -2100,14 +2262,20 @@
       <c r="E16" t="s">
         <v>49</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="G16" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G16" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>14</v>
       </c>
@@ -2123,14 +2291,20 @@
       <c r="E17" t="s">
         <v>52</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="G17" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G17" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>15</v>
       </c>
@@ -2146,14 +2320,20 @@
       <c r="E18" t="s">
         <v>55</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="G18" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G18" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>16</v>
       </c>
@@ -2169,14 +2349,20 @@
       <c r="E19" t="s">
         <v>58</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="G19" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G19" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>17</v>
       </c>
@@ -2192,14 +2378,20 @@
       <c r="E20" t="s">
         <v>61</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="G20" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G20" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>18</v>
       </c>
@@ -2215,14 +2407,20 @@
       <c r="E21" t="s">
         <v>64</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="5" t="s">
         <v>340</v>
       </c>
-      <c r="G21" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G21" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>19</v>
       </c>
@@ -2238,14 +2436,20 @@
       <c r="E22" t="s">
         <v>67</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="G22" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G22" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>20</v>
       </c>
@@ -2261,14 +2465,20 @@
       <c r="E23" t="s">
         <v>70</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="G23" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G23" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>21</v>
       </c>
@@ -2284,14 +2494,20 @@
       <c r="E24" t="s">
         <v>73</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="G24" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G24" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>22</v>
       </c>
@@ -2307,14 +2523,20 @@
       <c r="E25" t="s">
         <v>76</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="G25" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G25" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>23</v>
       </c>
@@ -2330,14 +2552,20 @@
       <c r="E26" t="s">
         <v>79</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="G26" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G26" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>24</v>
       </c>
@@ -2353,14 +2581,20 @@
       <c r="E27" t="s">
         <v>82</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="5" t="s">
         <v>346</v>
       </c>
-      <c r="G27" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G27" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>25</v>
       </c>
@@ -2376,14 +2610,20 @@
       <c r="E28" t="s">
         <v>85</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="G28" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G28" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>26</v>
       </c>
@@ -2399,14 +2639,20 @@
       <c r="E29" t="s">
         <v>88</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="G29" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G29" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>27</v>
       </c>
@@ -2422,14 +2668,20 @@
       <c r="E30" t="s">
         <v>91</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="G30" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G30" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>28</v>
       </c>
@@ -2445,14 +2697,20 @@
       <c r="E31" t="s">
         <v>94</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="G31" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G31" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>29</v>
       </c>
@@ -2468,14 +2726,20 @@
       <c r="E32" t="s">
         <v>97</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="G32" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G32" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>30</v>
       </c>
@@ -2491,14 +2755,20 @@
       <c r="E33" t="s">
         <v>100</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="G33" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G33" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>31</v>
       </c>
@@ -2514,14 +2784,20 @@
       <c r="E34" t="s">
         <v>103</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="G34" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G34" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>32</v>
       </c>
@@ -2537,14 +2813,20 @@
       <c r="E35" t="s">
         <v>106</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="5" t="s">
         <v>354</v>
       </c>
-      <c r="G35" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G35" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>33</v>
       </c>
@@ -2560,14 +2842,20 @@
       <c r="E36" t="s">
         <v>109</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F36" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="G36" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G36" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>34</v>
       </c>
@@ -2583,14 +2871,20 @@
       <c r="E37" t="s">
         <v>112</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="5" t="s">
         <v>356</v>
       </c>
-      <c r="G37" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G37" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>35</v>
       </c>
@@ -2606,14 +2900,20 @@
       <c r="E38" t="s">
         <v>115</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="5" t="s">
         <v>357</v>
       </c>
-      <c r="G38" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G38" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>36</v>
       </c>
@@ -2629,14 +2929,20 @@
       <c r="E39" t="s">
         <v>118</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="G39" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G39" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>37</v>
       </c>
@@ -2652,14 +2958,20 @@
       <c r="E40" t="s">
         <v>121</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F40" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="G40" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G40" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>38</v>
       </c>
@@ -2675,14 +2987,20 @@
       <c r="E41" t="s">
         <v>124</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F41" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="G41" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G41" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>39</v>
       </c>
@@ -2698,14 +3016,20 @@
       <c r="E42" t="s">
         <v>127</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F42" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="G42" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G42" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="I42" s="6" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>40</v>
       </c>
@@ -2721,14 +3045,20 @@
       <c r="E43" t="s">
         <v>130</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F43" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="G43" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G43" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>41</v>
       </c>
@@ -2744,14 +3074,20 @@
       <c r="E44" t="s">
         <v>133</v>
       </c>
-      <c r="F44" t="s">
+      <c r="F44" s="5" t="s">
         <v>363</v>
       </c>
-      <c r="G44" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G44" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>42</v>
       </c>
@@ -2767,14 +3103,20 @@
       <c r="E45" t="s">
         <v>136</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F45" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="G45" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G45" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>43</v>
       </c>
@@ -2790,14 +3132,20 @@
       <c r="E46" t="s">
         <v>139</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="G46" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G46" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="I46" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>44</v>
       </c>
@@ -2813,14 +3161,20 @@
       <c r="E47" t="s">
         <v>142</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F47" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="G47" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G47" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>45</v>
       </c>
@@ -2836,14 +3190,20 @@
       <c r="E48" t="s">
         <v>145</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F48" s="5" t="s">
         <v>367</v>
       </c>
-      <c r="G48" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G48" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="I48" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>46</v>
       </c>
@@ -2859,14 +3219,20 @@
       <c r="E49" t="s">
         <v>148</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F49" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="G49" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G49" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="I49" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>47</v>
       </c>
@@ -2882,14 +3248,20 @@
       <c r="E50" t="s">
         <v>151</v>
       </c>
-      <c r="F50" t="s">
+      <c r="F50" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="G50" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G50" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="I50" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>48</v>
       </c>
@@ -2905,14 +3277,20 @@
       <c r="E51" t="s">
         <v>154</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F51" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="G51" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G51" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="I51" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>49</v>
       </c>
@@ -2928,14 +3306,20 @@
       <c r="E52" t="s">
         <v>157</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F52" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="G52" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G52" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>50</v>
       </c>
@@ -2951,14 +3335,20 @@
       <c r="E53" t="s">
         <v>160</v>
       </c>
-      <c r="F53" t="s">
+      <c r="F53" s="5" t="s">
         <v>372</v>
       </c>
-      <c r="G53" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G53" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="I53" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>51</v>
       </c>
@@ -2974,14 +3364,20 @@
       <c r="E54" t="s">
         <v>163</v>
       </c>
-      <c r="F54" t="s">
+      <c r="F54" s="5" t="s">
         <v>373</v>
       </c>
-      <c r="G54" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G54" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="I54" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>52</v>
       </c>
@@ -2997,14 +3393,20 @@
       <c r="E55" t="s">
         <v>166</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F55" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="G55" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G55" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>53</v>
       </c>
@@ -3020,14 +3422,20 @@
       <c r="E56" t="s">
         <v>169</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F56" s="5" t="s">
         <v>375</v>
       </c>
-      <c r="G56" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G56" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="I56" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>54</v>
       </c>
@@ -3043,14 +3451,20 @@
       <c r="E57" t="s">
         <v>172</v>
       </c>
-      <c r="F57" t="s">
+      <c r="F57" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="G57" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G57" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H57" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="I57" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>55</v>
       </c>
@@ -3066,14 +3480,20 @@
       <c r="E58" t="s">
         <v>175</v>
       </c>
-      <c r="F58" t="s">
+      <c r="F58" s="5" t="s">
         <v>377</v>
       </c>
-      <c r="G58" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G58" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I58" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>56</v>
       </c>
@@ -3089,14 +3509,20 @@
       <c r="E59" t="s">
         <v>178</v>
       </c>
-      <c r="F59" t="s">
+      <c r="F59" s="5" t="s">
         <v>378</v>
       </c>
-      <c r="G59" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G59" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="I59" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>57</v>
       </c>
@@ -3112,14 +3538,20 @@
       <c r="E60" t="s">
         <v>181</v>
       </c>
-      <c r="F60" t="s">
+      <c r="F60" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="G60" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G60" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="I60" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>58</v>
       </c>
@@ -3135,14 +3567,20 @@
       <c r="E61" t="s">
         <v>184</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F61" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="G61" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G61" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="H61" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="I61" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>59</v>
       </c>
@@ -3158,14 +3596,20 @@
       <c r="E62" t="s">
         <v>187</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F62" s="5" t="s">
         <v>381</v>
       </c>
-      <c r="G62" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G62" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H62" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="I62" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>60</v>
       </c>
@@ -3181,14 +3625,20 @@
       <c r="E63" t="s">
         <v>190</v>
       </c>
-      <c r="F63" t="s">
+      <c r="F63" s="5" t="s">
         <v>382</v>
       </c>
-      <c r="G63" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G63" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="H63" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="I63" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>61</v>
       </c>
@@ -3204,14 +3654,20 @@
       <c r="E64" t="s">
         <v>193</v>
       </c>
-      <c r="F64" t="s">
+      <c r="F64" s="5" t="s">
         <v>383</v>
       </c>
-      <c r="G64" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G64" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="H64" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="I64" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>62</v>
       </c>
@@ -3227,14 +3683,20 @@
       <c r="E65" t="s">
         <v>196</v>
       </c>
-      <c r="F65" t="s">
+      <c r="F65" s="5" t="s">
         <v>384</v>
       </c>
-      <c r="G65" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G65" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H65" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="I65" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>63</v>
       </c>
@@ -3250,14 +3712,20 @@
       <c r="E66" t="s">
         <v>199</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F66" s="5" t="s">
         <v>385</v>
       </c>
-      <c r="G66" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G66" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="I66" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>64</v>
       </c>
@@ -3273,14 +3741,20 @@
       <c r="E67" t="s">
         <v>202</v>
       </c>
-      <c r="F67" t="s">
+      <c r="F67" s="5" t="s">
         <v>386</v>
       </c>
-      <c r="G67" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G67" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="H67" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="I67" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>65</v>
       </c>
@@ -3296,14 +3770,20 @@
       <c r="E68" t="s">
         <v>205</v>
       </c>
-      <c r="F68" t="s">
+      <c r="F68" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="G68" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G68" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="I68" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>66</v>
       </c>
@@ -3319,14 +3799,20 @@
       <c r="E69" t="s">
         <v>208</v>
       </c>
-      <c r="F69" t="s">
+      <c r="F69" s="5" t="s">
         <v>388</v>
       </c>
-      <c r="G69" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G69" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="I69" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>67</v>
       </c>
@@ -3342,14 +3828,20 @@
       <c r="E70" t="s">
         <v>211</v>
       </c>
-      <c r="F70" t="s">
+      <c r="F70" s="5" t="s">
         <v>389</v>
       </c>
-      <c r="G70" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G70" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="I70" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>68</v>
       </c>
@@ -3365,14 +3857,20 @@
       <c r="E71" t="s">
         <v>214</v>
       </c>
-      <c r="F71" t="s">
+      <c r="F71" s="5" t="s">
         <v>390</v>
       </c>
-      <c r="G71" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G71" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H71" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="I71" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>69</v>
       </c>
@@ -3388,14 +3886,20 @@
       <c r="E72" t="s">
         <v>217</v>
       </c>
-      <c r="F72" t="s">
+      <c r="F72" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="G72" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G72" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="I72" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>70</v>
       </c>
@@ -3411,14 +3915,20 @@
       <c r="E73" t="s">
         <v>220</v>
       </c>
-      <c r="F73" t="s">
-        <v>392</v>
-      </c>
-      <c r="G73" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F73" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="G73" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H73" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="I73" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>71</v>
       </c>
@@ -3434,14 +3944,20 @@
       <c r="E74" t="s">
         <v>223</v>
       </c>
-      <c r="F74" t="s">
-        <v>393</v>
-      </c>
-      <c r="G74" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F74" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="I74" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>72</v>
       </c>
@@ -3457,14 +3973,20 @@
       <c r="E75" t="s">
         <v>226</v>
       </c>
-      <c r="F75" t="s">
-        <v>394</v>
-      </c>
-      <c r="G75" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F75" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="G75" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H75" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="I75" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>73</v>
       </c>
@@ -3480,14 +4002,20 @@
       <c r="E76" t="s">
         <v>229</v>
       </c>
-      <c r="F76" t="s">
-        <v>395</v>
-      </c>
-      <c r="G76" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F76" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="G76" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H76" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="I76" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>74</v>
       </c>
@@ -3503,14 +4031,20 @@
       <c r="E77" t="s">
         <v>232</v>
       </c>
-      <c r="F77" t="s">
-        <v>396</v>
-      </c>
-      <c r="G77" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F77" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="G77" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H77" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="I77" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>75</v>
       </c>
@@ -3526,14 +4060,20 @@
       <c r="E78" t="s">
         <v>235</v>
       </c>
-      <c r="F78" t="s">
-        <v>397</v>
-      </c>
-      <c r="G78" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F78" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="G78" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="H78" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="I78" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>76</v>
       </c>
@@ -3549,14 +4089,20 @@
       <c r="E79" t="s">
         <v>238</v>
       </c>
-      <c r="F79" t="s">
-        <v>398</v>
-      </c>
-      <c r="G79" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F79" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="G79" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="I79" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>77</v>
       </c>
@@ -3572,14 +4118,20 @@
       <c r="E80" t="s">
         <v>241</v>
       </c>
-      <c r="F80" t="s">
-        <v>399</v>
-      </c>
-      <c r="G80" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F80" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="G80" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H80" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="I80" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>78</v>
       </c>
@@ -3595,14 +4147,20 @@
       <c r="E81" t="s">
         <v>244</v>
       </c>
-      <c r="F81" t="s">
-        <v>400</v>
-      </c>
-      <c r="G81" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F81" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="G81" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H81" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>79</v>
       </c>
@@ -3618,14 +4176,20 @@
       <c r="E82" t="s">
         <v>247</v>
       </c>
-      <c r="F82" t="s">
-        <v>420</v>
-      </c>
-      <c r="G82" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F82" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="G82" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H82" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="I82" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>80</v>
       </c>
@@ -3641,14 +4205,20 @@
       <c r="E83" t="s">
         <v>250</v>
       </c>
-      <c r="F83" t="s">
-        <v>401</v>
-      </c>
-      <c r="G83" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F83" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="H83" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="I83" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>81</v>
       </c>
@@ -3664,14 +4234,20 @@
       <c r="E84" t="s">
         <v>253</v>
       </c>
-      <c r="F84" t="s">
-        <v>402</v>
-      </c>
-      <c r="G84" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F84" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="G84" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="I84" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>82</v>
       </c>
@@ -3687,14 +4263,20 @@
       <c r="E85" t="s">
         <v>256</v>
       </c>
-      <c r="F85" t="s">
-        <v>403</v>
-      </c>
-      <c r="G85" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F85" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="G85" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="H85" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="I85" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>83</v>
       </c>
@@ -3710,14 +4292,20 @@
       <c r="E86" t="s">
         <v>259</v>
       </c>
-      <c r="F86" t="s">
-        <v>404</v>
-      </c>
-      <c r="G86" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F86" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="G86" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="H86" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="I86" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>84</v>
       </c>
@@ -3733,14 +4321,20 @@
       <c r="E87" t="s">
         <v>262</v>
       </c>
-      <c r="F87" t="s">
-        <v>405</v>
-      </c>
-      <c r="G87" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F87" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="G87" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H87" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="I87" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>85</v>
       </c>
@@ -3756,14 +4350,20 @@
       <c r="E88" t="s">
         <v>265</v>
       </c>
-      <c r="F88" t="s">
-        <v>406</v>
-      </c>
-      <c r="G88" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F88" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="G88" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H88" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="I88" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>86</v>
       </c>
@@ -3779,14 +4379,20 @@
       <c r="E89" t="s">
         <v>268</v>
       </c>
-      <c r="F89" t="s">
-        <v>407</v>
-      </c>
-      <c r="G89" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F89" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="G89" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H89" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="I89" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>87</v>
       </c>
@@ -3802,14 +4408,20 @@
       <c r="E90" t="s">
         <v>271</v>
       </c>
-      <c r="F90" t="s">
-        <v>408</v>
-      </c>
-      <c r="G90" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F90" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="G90" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H90" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="I90" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>88</v>
       </c>
@@ -3825,14 +4437,20 @@
       <c r="E91" t="s">
         <v>274</v>
       </c>
-      <c r="F91" t="s">
-        <v>409</v>
-      </c>
-      <c r="G91" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F91" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="G91" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H91" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I91" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>89</v>
       </c>
@@ -3848,14 +4466,20 @@
       <c r="E92" t="s">
         <v>277</v>
       </c>
-      <c r="F92" t="s">
-        <v>410</v>
-      </c>
-      <c r="G92" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F92" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="G92" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H92" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I92" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>90</v>
       </c>
@@ -3871,14 +4495,20 @@
       <c r="E93" t="s">
         <v>280</v>
       </c>
-      <c r="F93" t="s">
-        <v>411</v>
-      </c>
-      <c r="G93" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F93" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="G93" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H93" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I93" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>91</v>
       </c>
@@ -3894,14 +4524,20 @@
       <c r="E94" t="s">
         <v>283</v>
       </c>
-      <c r="F94" t="s">
-        <v>425</v>
-      </c>
-      <c r="G94" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F94" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="G94" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H94" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I94" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>92</v>
       </c>
@@ -3917,14 +4553,20 @@
       <c r="E95" t="s">
         <v>286</v>
       </c>
-      <c r="F95" t="s">
-        <v>431</v>
-      </c>
-      <c r="G95" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F95" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="G95" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H95" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I95" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>93</v>
       </c>
@@ -3940,14 +4582,20 @@
       <c r="E96" t="s">
         <v>289</v>
       </c>
-      <c r="F96" t="s">
-        <v>412</v>
-      </c>
-      <c r="G96" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F96" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="G96" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H96" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I96" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>94</v>
       </c>
@@ -3963,14 +4611,20 @@
       <c r="E97" t="s">
         <v>292</v>
       </c>
-      <c r="F97" t="s">
-        <v>413</v>
-      </c>
-      <c r="G97" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F97" s="5" t="s">
+        <v>412</v>
+      </c>
+      <c r="G97" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H97" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I97" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>95</v>
       </c>
@@ -3986,14 +4640,20 @@
       <c r="E98" t="s">
         <v>295</v>
       </c>
-      <c r="F98" t="s">
-        <v>414</v>
-      </c>
-      <c r="G98" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F98" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="G98" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H98" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I98" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>96</v>
       </c>
@@ -4009,14 +4669,20 @@
       <c r="E99" t="s">
         <v>298</v>
       </c>
-      <c r="F99" t="s">
-        <v>415</v>
-      </c>
-      <c r="G99" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F99" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="G99" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H99" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I99" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>97</v>
       </c>
@@ -4032,14 +4698,20 @@
       <c r="E100" t="s">
         <v>301</v>
       </c>
-      <c r="F100" t="s">
-        <v>421</v>
-      </c>
-      <c r="G100" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F100" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="G100" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H100" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I100" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>98</v>
       </c>
@@ -4055,14 +4727,20 @@
       <c r="E101" t="s">
         <v>304</v>
       </c>
-      <c r="F101" t="s">
-        <v>416</v>
-      </c>
-      <c r="G101" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F101" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="G101" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H101" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I101" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>99</v>
       </c>
@@ -4078,14 +4756,20 @@
       <c r="E102" t="s">
         <v>307</v>
       </c>
-      <c r="F102" t="s">
-        <v>417</v>
-      </c>
-      <c r="G102" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F102" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="G102" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H102" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I102" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>100</v>
       </c>
@@ -4101,14 +4785,20 @@
       <c r="E103" t="s">
         <v>310</v>
       </c>
-      <c r="F103" t="s">
-        <v>418</v>
-      </c>
-      <c r="G103" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F103" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="G103" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H103" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I103" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>101</v>
       </c>
@@ -4124,14 +4814,20 @@
       <c r="E104" t="s">
         <v>313</v>
       </c>
-      <c r="F104" t="s">
-        <v>430</v>
-      </c>
-      <c r="G104" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F104" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="G104" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H104" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I104" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>102</v>
       </c>
@@ -4147,14 +4843,20 @@
       <c r="E105" t="s">
         <v>316</v>
       </c>
-      <c r="F105" t="s">
-        <v>423</v>
-      </c>
-      <c r="G105" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F105" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="G105" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H105" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I105" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>103</v>
       </c>
@@ -4170,14 +4872,20 @@
       <c r="E106" t="s">
         <v>319</v>
       </c>
-      <c r="F106" t="s">
-        <v>422</v>
-      </c>
-      <c r="G106" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F106" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="G106" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H106" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I106" s="6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>104</v>
       </c>
@@ -4193,11 +4901,17 @@
       <c r="E107" t="s">
         <v>322</v>
       </c>
-      <c r="F107" t="s">
-        <v>424</v>
-      </c>
-      <c r="G107" t="s">
-        <v>427</v>
+      <c r="F107" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="G107" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="H107" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="I107" s="6" t="s">
+        <v>446</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Stefano's labels on 200 sample
</commit_message>
<xml_diff>
--- a/interim/cluster_review.xlsx
+++ b/interim/cluster_review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ilya/spatial-queries/interim/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D127EA7-7E40-CB40-BAEA-840E357689BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019A7E26-1D29-9A4D-8847-D54F03B01406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="26900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="26680" yWindow="620" windowWidth="24540" windowHeight="26900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -991,6 +991,9 @@
     <t>['what county is franktown colorado in', 'what county is harlowton mt in?', 'what county is plymouth washington in', 'white swan wa is in what county', 'what county is tukwila', 'what county is halliday nd in', 'what county is walla walla wa in', 'what county is spearfish sd in', 'what county is sibley, nd in?', 'which county is hayford ca']</t>
   </si>
   <si>
+    <t>Noise</t>
+  </si>
+  <si>
     <t>Area codes</t>
   </si>
   <si>
@@ -1241,9 +1244,6 @@
   </si>
   <si>
     <t>Biographical</t>
-  </si>
-  <si>
-    <t>Other</t>
   </si>
   <si>
     <t>Administrative</t>
@@ -1720,10 +1720,10 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -1743,7 +1743,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>407</v>
+        <v>323</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -1763,7 +1763,7 @@
         <v>10</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>408</v>
@@ -1786,7 +1786,7 @@
         <v>13</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>408</v>
@@ -1809,7 +1809,7 @@
         <v>16</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>421</v>
@@ -1832,7 +1832,7 @@
         <v>19</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>412</v>
@@ -1855,7 +1855,7 @@
         <v>22</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>422</v>
@@ -1878,7 +1878,7 @@
         <v>25</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>408</v>
@@ -1924,7 +1924,7 @@
         <v>31</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>411</v>
@@ -1947,7 +1947,7 @@
         <v>34</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>409</v>
@@ -1973,7 +1973,7 @@
         <v>416</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1996,7 +1996,7 @@
         <v>415</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -2016,7 +2016,7 @@
         <v>43</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>412</v>
@@ -2039,7 +2039,7 @@
         <v>46</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>414</v>
@@ -2062,7 +2062,7 @@
         <v>49</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G16" s="4" t="s">
         <v>408</v>
@@ -2085,7 +2085,7 @@
         <v>52</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>422</v>
@@ -2108,7 +2108,7 @@
         <v>55</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>412</v>
@@ -2131,7 +2131,7 @@
         <v>58</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G19" s="4" t="s">
         <v>414</v>
@@ -2154,7 +2154,7 @@
         <v>61</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>414</v>
@@ -2177,7 +2177,7 @@
         <v>64</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>421</v>
@@ -2200,7 +2200,7 @@
         <v>67</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>408</v>
@@ -2223,7 +2223,7 @@
         <v>70</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>421</v>
@@ -2246,7 +2246,7 @@
         <v>73</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G24" s="4" t="s">
         <v>421</v>
@@ -2269,7 +2269,7 @@
         <v>76</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G25" s="4" t="s">
         <v>414</v>
@@ -2292,7 +2292,7 @@
         <v>79</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G26" s="4" t="s">
         <v>414</v>
@@ -2315,7 +2315,7 @@
         <v>82</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>410</v>
@@ -2338,7 +2338,7 @@
         <v>85</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G28" s="4" t="s">
         <v>414</v>
@@ -2361,7 +2361,7 @@
         <v>88</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G29" s="4" t="s">
         <v>414</v>
@@ -2384,7 +2384,7 @@
         <v>91</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G30" s="4" t="s">
         <v>414</v>
@@ -2407,7 +2407,7 @@
         <v>94</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>414</v>
@@ -2430,7 +2430,7 @@
         <v>97</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G32" s="4" t="s">
         <v>414</v>
@@ -2453,7 +2453,7 @@
         <v>100</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G33" s="4" t="s">
         <v>409</v>
@@ -2476,7 +2476,7 @@
         <v>103</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G34" s="4" t="s">
         <v>409</v>
@@ -2499,7 +2499,7 @@
         <v>106</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G35" s="4" t="s">
         <v>421</v>
@@ -2522,7 +2522,7 @@
         <v>109</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G36" s="4" t="s">
         <v>414</v>
@@ -2545,7 +2545,7 @@
         <v>112</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G37" s="4" t="s">
         <v>410</v>
@@ -2568,7 +2568,7 @@
         <v>115</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G38" s="4" t="s">
         <v>414</v>
@@ -2591,7 +2591,7 @@
         <v>118</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G39" s="4" t="s">
         <v>414</v>
@@ -2614,7 +2614,7 @@
         <v>121</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G40" s="4" t="s">
         <v>414</v>
@@ -2637,10 +2637,10 @@
         <v>124</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -2660,7 +2660,7 @@
         <v>127</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="G42" s="4" t="s">
         <v>422</v>
@@ -2683,7 +2683,7 @@
         <v>130</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G43" s="4" t="s">
         <v>412</v>
@@ -2706,7 +2706,7 @@
         <v>133</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G44" s="4" t="s">
         <v>412</v>
@@ -2775,7 +2775,7 @@
         <v>142</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G47" s="4" t="s">
         <v>409</v>
@@ -2798,7 +2798,7 @@
         <v>145</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G48" s="4" t="s">
         <v>409</v>
@@ -2844,7 +2844,7 @@
         <v>151</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G50" s="4" t="s">
         <v>414</v>
@@ -2867,7 +2867,7 @@
         <v>154</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G51" s="4" t="s">
         <v>414</v>
@@ -2890,7 +2890,7 @@
         <v>157</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G52" s="4" t="s">
         <v>410</v>
@@ -2913,7 +2913,7 @@
         <v>160</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G53" s="4" t="s">
         <v>410</v>
@@ -2936,7 +2936,7 @@
         <v>163</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G54" s="4" t="s">
         <v>411</v>
@@ -2959,7 +2959,7 @@
         <v>166</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G55" s="4" t="s">
         <v>411</v>
@@ -2982,7 +2982,7 @@
         <v>169</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G56" s="4" t="s">
         <v>410</v>
@@ -3005,7 +3005,7 @@
         <v>172</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G57" s="4" t="s">
         <v>410</v>
@@ -3028,7 +3028,7 @@
         <v>175</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G58" s="4" t="s">
         <v>408</v>
@@ -3051,7 +3051,7 @@
         <v>178</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="G59" s="4" t="s">
         <v>409</v>
@@ -3074,7 +3074,7 @@
         <v>181</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G60" s="4" t="s">
         <v>409</v>
@@ -3097,7 +3097,7 @@
         <v>184</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G61" s="4" t="s">
         <v>409</v>
@@ -3120,7 +3120,7 @@
         <v>187</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G62" s="4" t="s">
         <v>411</v>
@@ -3143,7 +3143,7 @@
         <v>190</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="G63" s="4" t="s">
         <v>412</v>
@@ -3166,7 +3166,7 @@
         <v>193</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G64" s="4" t="s">
         <v>412</v>
@@ -3189,7 +3189,7 @@
         <v>196</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G65" s="4" t="s">
         <v>410</v>
@@ -3212,7 +3212,7 @@
         <v>199</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G66" s="4" t="s">
         <v>410</v>
@@ -3235,7 +3235,7 @@
         <v>202</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G67" s="4" t="s">
         <v>412</v>
@@ -3258,7 +3258,7 @@
         <v>205</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G68" s="4" t="s">
         <v>411</v>
@@ -3281,7 +3281,7 @@
         <v>208</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G69" s="4" t="s">
         <v>410</v>
@@ -3304,7 +3304,7 @@
         <v>211</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G70" s="4" t="s">
         <v>410</v>
@@ -3327,7 +3327,7 @@
         <v>214</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="G71" s="4" t="s">
         <v>411</v>
@@ -3350,7 +3350,7 @@
         <v>217</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G72" s="4" t="s">
         <v>409</v>
@@ -3396,7 +3396,7 @@
         <v>223</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G74" s="4" t="s">
         <v>410</v>
@@ -3419,7 +3419,7 @@
         <v>226</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G75" s="4" t="s">
         <v>410</v>
@@ -3442,7 +3442,7 @@
         <v>229</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G76" s="4" t="s">
         <v>410</v>
@@ -3465,7 +3465,7 @@
         <v>232</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="G77" s="4" t="s">
         <v>410</v>
@@ -3488,7 +3488,7 @@
         <v>235</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G78" s="4" t="s">
         <v>410</v>
@@ -3511,7 +3511,7 @@
         <v>238</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G79" s="4" t="s">
         <v>408</v>
@@ -3534,7 +3534,7 @@
         <v>241</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G80" s="4" t="s">
         <v>408</v>
@@ -3557,7 +3557,7 @@
         <v>244</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G81" s="4" t="s">
         <v>411</v>
@@ -3580,7 +3580,7 @@
         <v>247</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G82" s="4" t="s">
         <v>411</v>
@@ -3603,7 +3603,7 @@
         <v>250</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G83" s="4" t="s">
         <v>410</v>
@@ -3626,7 +3626,7 @@
         <v>253</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G84" s="4" t="s">
         <v>410</v>
@@ -3649,7 +3649,7 @@
         <v>256</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="G85" s="4" t="s">
         <v>410</v>
@@ -3672,7 +3672,7 @@
         <v>259</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G86" s="4" t="s">
         <v>410</v>
@@ -3695,7 +3695,7 @@
         <v>262</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G87" s="4" t="s">
         <v>411</v>
@@ -3718,7 +3718,7 @@
         <v>265</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G88" s="4" t="s">
         <v>411</v>
@@ -3741,7 +3741,7 @@
         <v>268</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="G89" s="4" t="s">
         <v>411</v>
@@ -3764,7 +3764,7 @@
         <v>271</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G90" s="4" t="s">
         <v>411</v>
@@ -3787,7 +3787,7 @@
         <v>274</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G91" s="4" t="s">
         <v>408</v>
@@ -3810,7 +3810,7 @@
         <v>277</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G92" s="4" t="s">
         <v>408</v>
@@ -3833,7 +3833,7 @@
         <v>280</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G93" s="4" t="s">
         <v>408</v>
@@ -3856,7 +3856,7 @@
         <v>283</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G94" s="4" t="s">
         <v>408</v>
@@ -3879,7 +3879,7 @@
         <v>286</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G95" s="4" t="s">
         <v>408</v>
@@ -3902,7 +3902,7 @@
         <v>289</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G96" s="4" t="s">
         <v>408</v>
@@ -3925,7 +3925,7 @@
         <v>292</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G97" s="4" t="s">
         <v>408</v>
@@ -3948,7 +3948,7 @@
         <v>295</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G98" s="4" t="s">
         <v>408</v>
@@ -3971,7 +3971,7 @@
         <v>298</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G99" s="4" t="s">
         <v>408</v>
@@ -3994,7 +3994,7 @@
         <v>301</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G100" s="4" t="s">
         <v>408</v>
@@ -4017,7 +4017,7 @@
         <v>304</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G101" s="4" t="s">
         <v>408</v>
@@ -4040,7 +4040,7 @@
         <v>307</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G102" s="4" t="s">
         <v>408</v>
@@ -4063,7 +4063,7 @@
         <v>310</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G103" s="4" t="s">
         <v>408</v>
@@ -4086,7 +4086,7 @@
         <v>313</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G104" s="4" t="s">
         <v>408</v>
@@ -4109,7 +4109,7 @@
         <v>316</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G105" s="4" t="s">
         <v>408</v>
@@ -4132,7 +4132,7 @@
         <v>319</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G106" s="4" t="s">
         <v>408</v>
@@ -4155,7 +4155,7 @@
         <v>322</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G107" s="4" t="s">
         <v>408</v>

</xml_diff>